<commit_message>
Add live betting odds integration and enhanced recommendations
- Add OddsFetcher class for fetching live betting odds from The Odds API
- Implement enhanced recommendations component with value analysis
- Integrate betting odds with historical performance for value edge calculation
- Add sample odds data for testing without API key
- Create comprehensive betting odds guide
- Replace placeholder recommendations tab with full feature
- Support for tournament winner odds and value edge analysis
- Visual breakdowns with Plotly charts
</commit_message>
<xml_diff>
--- a/List of enhancements.xlsx
+++ b/List of enhancements.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://l48prod-my.sharepoint.com/personal/austin_wheeler_bpx_com/Documents/Documents/VS Code/PGA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="59" documentId="8_{66DCC003-5AF0-4C0F-881D-DB24B37DE8C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ED1AA1CF-D0A0-455B-8670-036B23B9B432}"/>
+  <xr:revisionPtr revIDLastSave="64" documentId="8_{66DCC003-5AF0-4C0F-881D-DB24B37DE8C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A68603E9-38BB-42EF-907F-F2D10B7D91DF}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{7CDC0889-F374-43A9-B162-4F8D9DFD3995}"/>
+    <workbookView minimized="1" xWindow="2380" yWindow="2560" windowWidth="6870" windowHeight="11300" xr2:uid="{7CDC0889-F374-43A9-B162-4F8D9DFD3995}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -50,13 +50,13 @@
     <t>Can I pull betting odds into the analysis and display in the table on the In the Field section, this would include odds to win and odds to make top 10</t>
   </si>
   <si>
-    <t>How do I publish this to the web so I can share with my family and friends but not have just anyone access it.</t>
-  </si>
-  <si>
     <t>Lets pull more data all the way back to 2000 along with earnings data. After we pull all this data we need to implement the same Tournament name aggregation we did for the 2020-2025 data.</t>
   </si>
   <si>
     <t>Option to manually input the Value calc % for each piece of calc</t>
+  </si>
+  <si>
+    <t>Use the old data to train the model for the value number</t>
   </si>
 </sst>
 </file>
@@ -88,7 +88,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -111,27 +111,15 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -490,43 +478,43 @@
       <c r="A3" s="1">
         <v>1</v>
       </c>
-      <c r="B3" s="1"/>
+      <c r="B3" s="1" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>2</v>
       </c>
-      <c r="B4" s="4"/>
+      <c r="B4" s="1" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>3</v>
       </c>
-      <c r="B5" s="1"/>
+      <c r="B5" s="1" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>4</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>3</v>
-      </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>5</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>4</v>
+      <c r="B7" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>6</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>5</v>
-      </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
@@ -543,9 +531,6 @@
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>9</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>